<commit_message>
Completed more data about AAPL
</commit_message>
<xml_diff>
--- a/8. Template_Stock.xlsx
+++ b/8. Template_Stock.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/KINGSTON/MyStockData/Finance-StockLists/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B96E6F6-7D86-A749-8CCE-2FEAF77DD6BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FDB2352-A58B-A146-96F1-CDAF63DF4EA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="14400" xr2:uid="{AEC0C047-6E16-294C-82BD-58123BA913A1}"/>
   </bookViews>
@@ -116,33 +116,6 @@
 <file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
-    <author>tc={414A3395-9FE7-8D48-97C3-96B990240E0B}</author>
-    <author>tc={EFE71069-E88D-A343-BA5C-490270B76A85}</author>
-  </authors>
-  <commentList>
-    <comment ref="H18" authorId="0" shapeId="0" xr:uid="{414A3395-9FE7-8D48-97C3-96B990240E0B}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    Adjusted manually to exclude the one time tax income for FY 2025. extracted 22000 from the income before taxes</t>
-      </text>
-    </comment>
-    <comment ref="P18" authorId="1" shapeId="0" xr:uid="{EFE71069-E88D-A343-BA5C-490270B76A85}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    Set a manual value to exclude the one time tax income</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
     <author>tc={823E70A9-8202-AD4F-B27F-441FEEF6DACF}</author>
     <author>tc={15CC66A8-AFB4-7E4D-B1BB-80F7466557AC}</author>
   </authors>
@@ -167,7 +140,7 @@
 </comments>
 </file>
 
-<file path=xl/comments5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>tc={1C41E23C-4E49-DB45-AA4B-41462965580A}</author>
@@ -203,7 +176,7 @@
 </comments>
 </file>
 
-<file path=xl/comments6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments5.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>tc={FE7F7696-1DC8-8740-9551-F021B84F5B84}</author>
@@ -221,7 +194,7 @@
 </comments>
 </file>
 
-<file path=xl/comments7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments6.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>tc={3E138CA2-608A-1149-B0E7-AC81514F3EC2}</author>
@@ -2322,6 +2295,15 @@
     <xf numFmtId="165" fontId="24" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="10" fontId="18" fillId="8" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="3" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="13" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2338,15 +2320,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2378,6 +2351,9 @@
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Sheet1"/>
       <sheetName val="1. List_AutomaticData"/>
@@ -2741,17 +2717,6 @@
 
 <file path=xl/threadedComments/threadedComment3.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="H18" dT="2026-02-28T18:08:49.14" personId="{C1D857D3-F592-2946-8369-15D188CA547D}" id="{414A3395-9FE7-8D48-97C3-96B990240E0B}">
-    <text>Adjusted manually to exclude the one time tax income for FY 2025. extracted 22000 from the income before taxes</text>
-  </threadedComment>
-  <threadedComment ref="P18" dT="2026-02-28T18:16:06.49" personId="{C1D857D3-F592-2946-8369-15D188CA547D}" id="{EFE71069-E88D-A343-BA5C-490270B76A85}">
-    <text>Set a manual value to exclude the one time tax income</text>
-  </threadedComment>
-</ThreadedComments>
-</file>
-
-<file path=xl/threadedComments/threadedComment4.xml><?xml version="1.0" encoding="utf-8"?>
-<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <threadedComment ref="B38" dT="2026-02-18T19:50:02.62" personId="{C1D857D3-F592-2946-8369-15D188CA547D}" id="{823E70A9-8202-AD4F-B27F-441FEEF6DACF}">
     <text>Use the value from Avg useful life under Average useful life of PP&amp;E. Make the value slightly higher</text>
   </threadedComment>
@@ -2761,7 +2726,7 @@
 </ThreadedComments>
 </file>
 
-<file path=xl/threadedComments/threadedComment5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/threadedComments/threadedComment4.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <threadedComment ref="B16" dT="2026-02-19T19:30:25.86" personId="{C1D857D3-F592-2946-8369-15D188CA547D}" id="{1C41E23C-4E49-DB45-AA4B-41462965580A}">
     <text>Forecast values taken from the recent 10-K</text>
@@ -2775,7 +2740,7 @@
 </ThreadedComments>
 </file>
 
-<file path=xl/threadedComments/threadedComment6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/threadedComments/threadedComment5.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <threadedComment ref="B26" dT="2026-02-20T23:46:38.49" personId="{C1D857D3-F592-2946-8369-15D188CA547D}" id="{FE7F7696-1DC8-8740-9551-F021B84F5B84}">
     <text>The same growth rate as operating lease right of use assets</text>
@@ -2783,7 +2748,7 @@
 </ThreadedComments>
 </file>
 
-<file path=xl/threadedComments/threadedComment7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/threadedComments/threadedComment6.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <threadedComment ref="B9" dT="2026-02-28T14:18:18.18" personId="{C1D857D3-F592-2946-8369-15D188CA547D}" id="{3E138CA2-608A-1149-B0E7-AC81514F3EC2}">
     <text>10 year government bond yield</text>
@@ -2917,7 +2882,7 @@
         <v>325</v>
       </c>
       <c r="C15" s="20">
-        <f>C3*'Statement Q'!J116</f>
+        <f>C3*'Statement Q'!N116</f>
         <v>0</v>
       </c>
     </row>
@@ -3162,20 +3127,20 @@
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A5" s="103"/>
-      <c r="C5" s="220" t="s">
+      <c r="C5" s="223" t="s">
         <v>168</v>
       </c>
-      <c r="D5" s="220"/>
-      <c r="E5" s="220"/>
-      <c r="F5" s="220"/>
-      <c r="G5" s="223"/>
-      <c r="H5" s="224" t="s">
+      <c r="D5" s="223"/>
+      <c r="E5" s="223"/>
+      <c r="F5" s="223"/>
+      <c r="G5" s="226"/>
+      <c r="H5" s="227" t="s">
         <v>169</v>
       </c>
-      <c r="I5" s="220"/>
-      <c r="J5" s="220"/>
-      <c r="K5" s="220"/>
-      <c r="L5" s="220"/>
+      <c r="I5" s="223"/>
+      <c r="J5" s="223"/>
+      <c r="K5" s="223"/>
+      <c r="L5" s="223"/>
       <c r="P5" s="228"/>
       <c r="Q5" s="228"/>
       <c r="R5" s="228"/>
@@ -3193,18 +3158,18 @@
     <row r="7" spans="1:28" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="108"/>
       <c r="B7" s="92"/>
-      <c r="C7" s="219" t="s">
+      <c r="C7" s="222" t="s">
         <v>178</v>
       </c>
-      <c r="D7" s="219"/>
-      <c r="E7" s="219"/>
-      <c r="F7" s="219"/>
-      <c r="G7" s="219"/>
-      <c r="H7" s="219"/>
-      <c r="I7" s="219"/>
-      <c r="J7" s="219"/>
-      <c r="K7" s="219"/>
-      <c r="L7" s="219"/>
+      <c r="D7" s="222"/>
+      <c r="E7" s="222"/>
+      <c r="F7" s="222"/>
+      <c r="G7" s="222"/>
+      <c r="H7" s="222"/>
+      <c r="I7" s="222"/>
+      <c r="J7" s="222"/>
+      <c r="K7" s="222"/>
+      <c r="L7" s="222"/>
       <c r="P7" s="228"/>
       <c r="Q7" s="228"/>
       <c r="R7" s="228"/>
@@ -3342,18 +3307,18 @@
       <c r="N11" s="91"/>
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="C12" s="219" t="s">
+      <c r="C12" s="222" t="s">
         <v>24</v>
       </c>
-      <c r="D12" s="219"/>
-      <c r="E12" s="219"/>
-      <c r="F12" s="219"/>
-      <c r="G12" s="219"/>
-      <c r="H12" s="219"/>
-      <c r="I12" s="219"/>
-      <c r="J12" s="219"/>
-      <c r="K12" s="219"/>
-      <c r="L12" s="219"/>
+      <c r="D12" s="222"/>
+      <c r="E12" s="222"/>
+      <c r="F12" s="222"/>
+      <c r="G12" s="222"/>
+      <c r="H12" s="222"/>
+      <c r="I12" s="222"/>
+      <c r="J12" s="222"/>
+      <c r="K12" s="222"/>
+      <c r="L12" s="222"/>
       <c r="N12" s="91"/>
       <c r="P12" s="228"/>
       <c r="Q12" s="228"/>
@@ -3667,18 +3632,18 @@
       <c r="D18" s="20"/>
     </row>
     <row r="20" spans="2:28" x14ac:dyDescent="0.2">
-      <c r="C20" s="219" t="s">
+      <c r="C20" s="222" t="s">
         <v>226</v>
       </c>
-      <c r="D20" s="219"/>
-      <c r="E20" s="219"/>
-      <c r="F20" s="219"/>
-      <c r="G20" s="219"/>
-      <c r="H20" s="219"/>
-      <c r="I20" s="219"/>
-      <c r="J20" s="219"/>
-      <c r="K20" s="219"/>
-      <c r="L20" s="219"/>
+      <c r="D20" s="222"/>
+      <c r="E20" s="222"/>
+      <c r="F20" s="222"/>
+      <c r="G20" s="222"/>
+      <c r="H20" s="222"/>
+      <c r="I20" s="222"/>
+      <c r="J20" s="222"/>
+      <c r="K20" s="222"/>
+      <c r="L20" s="222"/>
     </row>
     <row r="21" spans="2:28" x14ac:dyDescent="0.2">
       <c r="B21" s="7" t="s">
@@ -3903,10 +3868,10 @@
       <c r="C27" s="228"/>
     </row>
     <row r="28" spans="2:28" x14ac:dyDescent="0.2">
-      <c r="B28" s="220" t="s">
+      <c r="B28" s="223" t="s">
         <v>249</v>
       </c>
-      <c r="C28" s="220"/>
+      <c r="C28" s="223"/>
     </row>
     <row r="29" spans="2:28" x14ac:dyDescent="0.2">
       <c r="B29" s="1" t="s">
@@ -3917,18 +3882,18 @@
       </c>
     </row>
     <row r="31" spans="2:28" x14ac:dyDescent="0.2">
-      <c r="C31" s="219" t="s">
+      <c r="C31" s="222" t="s">
         <v>250</v>
       </c>
-      <c r="D31" s="219"/>
-      <c r="E31" s="219"/>
-      <c r="F31" s="219"/>
-      <c r="G31" s="219"/>
-      <c r="H31" s="219"/>
-      <c r="I31" s="219"/>
-      <c r="J31" s="219"/>
-      <c r="K31" s="219"/>
-      <c r="L31" s="219"/>
+      <c r="D31" s="222"/>
+      <c r="E31" s="222"/>
+      <c r="F31" s="222"/>
+      <c r="G31" s="222"/>
+      <c r="H31" s="222"/>
+      <c r="I31" s="222"/>
+      <c r="J31" s="222"/>
+      <c r="K31" s="222"/>
+      <c r="L31" s="222"/>
     </row>
     <row r="32" spans="2:28" x14ac:dyDescent="0.2">
       <c r="B32" s="7" t="s">
@@ -4135,18 +4100,18 @@
       <c r="C40" s="228"/>
     </row>
     <row r="41" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="C41" s="219" t="s">
+      <c r="C41" s="222" t="s">
         <v>251</v>
       </c>
-      <c r="D41" s="219"/>
-      <c r="E41" s="219"/>
-      <c r="F41" s="219"/>
-      <c r="G41" s="219"/>
-      <c r="H41" s="219"/>
-      <c r="I41" s="219"/>
-      <c r="J41" s="219"/>
-      <c r="K41" s="219"/>
-      <c r="L41" s="219"/>
+      <c r="D41" s="222"/>
+      <c r="E41" s="222"/>
+      <c r="F41" s="222"/>
+      <c r="G41" s="222"/>
+      <c r="H41" s="222"/>
+      <c r="I41" s="222"/>
+      <c r="J41" s="222"/>
+      <c r="K41" s="222"/>
+      <c r="L41" s="222"/>
     </row>
     <row r="42" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B42" s="7" t="s">
@@ -4281,20 +4246,20 @@
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A3" s="103"/>
-      <c r="C3" s="220" t="s">
+      <c r="C3" s="223" t="s">
         <v>168</v>
       </c>
-      <c r="D3" s="220"/>
-      <c r="E3" s="220"/>
-      <c r="F3" s="220"/>
-      <c r="G3" s="223"/>
-      <c r="H3" s="224" t="s">
+      <c r="D3" s="223"/>
+      <c r="E3" s="223"/>
+      <c r="F3" s="223"/>
+      <c r="G3" s="226"/>
+      <c r="H3" s="227" t="s">
         <v>169</v>
       </c>
-      <c r="I3" s="220"/>
-      <c r="J3" s="220"/>
-      <c r="K3" s="220"/>
-      <c r="L3" s="220"/>
+      <c r="I3" s="223"/>
+      <c r="J3" s="223"/>
+      <c r="K3" s="223"/>
+      <c r="L3" s="223"/>
       <c r="P3" s="228"/>
       <c r="Q3" s="228"/>
       <c r="R3" s="228"/>
@@ -4312,18 +4277,18 @@
     <row r="5" spans="1:28" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="108"/>
       <c r="B5" s="92"/>
-      <c r="C5" s="219" t="s">
+      <c r="C5" s="222" t="s">
         <v>178</v>
       </c>
-      <c r="D5" s="219"/>
-      <c r="E5" s="219"/>
-      <c r="F5" s="219"/>
-      <c r="G5" s="219"/>
-      <c r="H5" s="219"/>
-      <c r="I5" s="219"/>
-      <c r="J5" s="219"/>
-      <c r="K5" s="219"/>
-      <c r="L5" s="219"/>
+      <c r="D5" s="222"/>
+      <c r="E5" s="222"/>
+      <c r="F5" s="222"/>
+      <c r="G5" s="222"/>
+      <c r="H5" s="222"/>
+      <c r="I5" s="222"/>
+      <c r="J5" s="222"/>
+      <c r="K5" s="222"/>
+      <c r="L5" s="222"/>
       <c r="P5" s="228"/>
       <c r="Q5" s="228"/>
       <c r="R5" s="228"/>
@@ -4579,18 +4544,18 @@
       <c r="N11" s="91"/>
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="C12" s="219" t="s">
+      <c r="C12" s="222" t="s">
         <v>237</v>
       </c>
-      <c r="D12" s="219"/>
-      <c r="E12" s="219"/>
-      <c r="F12" s="219"/>
-      <c r="G12" s="219"/>
-      <c r="H12" s="219"/>
-      <c r="I12" s="219"/>
-      <c r="J12" s="219"/>
-      <c r="K12" s="219"/>
-      <c r="L12" s="219"/>
+      <c r="D12" s="222"/>
+      <c r="E12" s="222"/>
+      <c r="F12" s="222"/>
+      <c r="G12" s="222"/>
+      <c r="H12" s="222"/>
+      <c r="I12" s="222"/>
+      <c r="J12" s="222"/>
+      <c r="K12" s="222"/>
+      <c r="L12" s="222"/>
       <c r="N12" s="91"/>
       <c r="P12" s="228"/>
       <c r="Q12" s="228"/>
@@ -4843,18 +4808,18 @@
       <c r="D17" s="20"/>
     </row>
     <row r="19" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="C19" s="219" t="s">
+      <c r="C19" s="222" t="s">
         <v>256</v>
       </c>
-      <c r="D19" s="219"/>
-      <c r="E19" s="219"/>
-      <c r="F19" s="219"/>
-      <c r="G19" s="219"/>
-      <c r="H19" s="219"/>
-      <c r="I19" s="219"/>
-      <c r="J19" s="219"/>
-      <c r="K19" s="219"/>
-      <c r="L19" s="219"/>
+      <c r="D19" s="222"/>
+      <c r="E19" s="222"/>
+      <c r="F19" s="222"/>
+      <c r="G19" s="222"/>
+      <c r="H19" s="222"/>
+      <c r="I19" s="222"/>
+      <c r="J19" s="222"/>
+      <c r="K19" s="222"/>
+      <c r="L19" s="222"/>
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B20" s="7" t="s">
@@ -5041,18 +5006,18 @@
       <c r="C25" s="228"/>
     </row>
     <row r="26" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="C26" s="219" t="s">
+      <c r="C26" s="222" t="s">
         <v>267</v>
       </c>
-      <c r="D26" s="219"/>
-      <c r="E26" s="219"/>
-      <c r="F26" s="219"/>
-      <c r="G26" s="219"/>
-      <c r="H26" s="219"/>
-      <c r="I26" s="219"/>
-      <c r="J26" s="219"/>
-      <c r="K26" s="219"/>
-      <c r="L26" s="219"/>
+      <c r="D26" s="222"/>
+      <c r="E26" s="222"/>
+      <c r="F26" s="222"/>
+      <c r="G26" s="222"/>
+      <c r="H26" s="222"/>
+      <c r="I26" s="222"/>
+      <c r="J26" s="222"/>
+      <c r="K26" s="222"/>
+      <c r="L26" s="222"/>
     </row>
     <row r="27" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B27" s="7" t="s">
@@ -5296,18 +5261,18 @@
       <c r="G33" s="143"/>
     </row>
     <row r="34" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="C34" s="219" t="s">
+      <c r="C34" s="222" t="s">
         <v>268</v>
       </c>
-      <c r="D34" s="219"/>
-      <c r="E34" s="219"/>
-      <c r="F34" s="219"/>
-      <c r="G34" s="219"/>
-      <c r="H34" s="219"/>
-      <c r="I34" s="219"/>
-      <c r="J34" s="219"/>
-      <c r="K34" s="219"/>
-      <c r="L34" s="219"/>
+      <c r="D34" s="222"/>
+      <c r="E34" s="222"/>
+      <c r="F34" s="222"/>
+      <c r="G34" s="222"/>
+      <c r="H34" s="222"/>
+      <c r="I34" s="222"/>
+      <c r="J34" s="222"/>
+      <c r="K34" s="222"/>
+      <c r="L34" s="222"/>
     </row>
     <row r="35" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B35" s="7" t="s">
@@ -5580,20 +5545,20 @@
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A3" s="103"/>
-      <c r="C3" s="220" t="s">
+      <c r="C3" s="223" t="s">
         <v>168</v>
       </c>
-      <c r="D3" s="220"/>
-      <c r="E3" s="220"/>
-      <c r="F3" s="220"/>
-      <c r="G3" s="223"/>
-      <c r="H3" s="224" t="s">
+      <c r="D3" s="223"/>
+      <c r="E3" s="223"/>
+      <c r="F3" s="223"/>
+      <c r="G3" s="226"/>
+      <c r="H3" s="227" t="s">
         <v>169</v>
       </c>
-      <c r="I3" s="220"/>
-      <c r="J3" s="220"/>
-      <c r="K3" s="220"/>
-      <c r="L3" s="220"/>
+      <c r="I3" s="223"/>
+      <c r="J3" s="223"/>
+      <c r="K3" s="223"/>
+      <c r="L3" s="223"/>
       <c r="P3" s="228"/>
       <c r="Q3" s="228"/>
       <c r="R3" s="228"/>
@@ -5611,18 +5576,18 @@
     <row r="5" spans="1:28" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="108"/>
       <c r="B5" s="92"/>
-      <c r="C5" s="219" t="s">
+      <c r="C5" s="222" t="s">
         <v>178</v>
       </c>
-      <c r="D5" s="219"/>
-      <c r="E5" s="219"/>
-      <c r="F5" s="219"/>
-      <c r="G5" s="219"/>
-      <c r="H5" s="219"/>
-      <c r="I5" s="219"/>
-      <c r="J5" s="219"/>
-      <c r="K5" s="219"/>
-      <c r="L5" s="219"/>
+      <c r="D5" s="222"/>
+      <c r="E5" s="222"/>
+      <c r="F5" s="222"/>
+      <c r="G5" s="222"/>
+      <c r="H5" s="222"/>
+      <c r="I5" s="222"/>
+      <c r="J5" s="222"/>
+      <c r="K5" s="222"/>
+      <c r="L5" s="222"/>
       <c r="P5" s="228"/>
       <c r="Q5" s="228"/>
       <c r="R5" s="228"/>
@@ -5938,18 +5903,18 @@
       <c r="C12" s="228"/>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="C13" s="219" t="s">
+      <c r="C13" s="222" t="s">
         <v>289</v>
       </c>
-      <c r="D13" s="219"/>
-      <c r="E13" s="219"/>
-      <c r="F13" s="219"/>
-      <c r="G13" s="219"/>
-      <c r="H13" s="219"/>
-      <c r="I13" s="219"/>
-      <c r="J13" s="219"/>
-      <c r="K13" s="219"/>
-      <c r="L13" s="219"/>
+      <c r="D13" s="222"/>
+      <c r="E13" s="222"/>
+      <c r="F13" s="222"/>
+      <c r="G13" s="222"/>
+      <c r="H13" s="222"/>
+      <c r="I13" s="222"/>
+      <c r="J13" s="222"/>
+      <c r="K13" s="222"/>
+      <c r="L13" s="222"/>
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B14" s="7" t="s">
@@ -6193,18 +6158,18 @@
       <c r="G20" s="143"/>
     </row>
     <row r="21" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="C21" s="219" t="s">
+      <c r="C21" s="222" t="s">
         <v>268</v>
       </c>
-      <c r="D21" s="219"/>
-      <c r="E21" s="219"/>
-      <c r="F21" s="219"/>
-      <c r="G21" s="219"/>
-      <c r="H21" s="219"/>
-      <c r="I21" s="219"/>
-      <c r="J21" s="219"/>
-      <c r="K21" s="219"/>
-      <c r="L21" s="219"/>
+      <c r="D21" s="222"/>
+      <c r="E21" s="222"/>
+      <c r="F21" s="222"/>
+      <c r="G21" s="222"/>
+      <c r="H21" s="222"/>
+      <c r="I21" s="222"/>
+      <c r="J21" s="222"/>
+      <c r="K21" s="222"/>
+      <c r="L21" s="222"/>
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B22" s="7" t="s">
@@ -6493,20 +6458,20 @@
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A3" s="103"/>
-      <c r="C3" s="220" t="s">
+      <c r="C3" s="223" t="s">
         <v>168</v>
       </c>
-      <c r="D3" s="220"/>
-      <c r="E3" s="220"/>
-      <c r="F3" s="220"/>
-      <c r="G3" s="223"/>
-      <c r="H3" s="224" t="s">
+      <c r="D3" s="223"/>
+      <c r="E3" s="223"/>
+      <c r="F3" s="223"/>
+      <c r="G3" s="226"/>
+      <c r="H3" s="227" t="s">
         <v>169</v>
       </c>
-      <c r="I3" s="220"/>
-      <c r="J3" s="220"/>
-      <c r="K3" s="220"/>
-      <c r="L3" s="220"/>
+      <c r="I3" s="223"/>
+      <c r="J3" s="223"/>
+      <c r="K3" s="223"/>
+      <c r="L3" s="223"/>
       <c r="P3" s="228"/>
       <c r="Q3" s="228"/>
       <c r="R3" s="228"/>
@@ -6524,18 +6489,18 @@
     <row r="5" spans="1:28" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="108"/>
       <c r="B5" s="92"/>
-      <c r="C5" s="219" t="s">
+      <c r="C5" s="222" t="s">
         <v>301</v>
       </c>
-      <c r="D5" s="219"/>
-      <c r="E5" s="219"/>
-      <c r="F5" s="219"/>
-      <c r="G5" s="219"/>
-      <c r="H5" s="219"/>
-      <c r="I5" s="219"/>
-      <c r="J5" s="219"/>
-      <c r="K5" s="219"/>
-      <c r="L5" s="219"/>
+      <c r="D5" s="222"/>
+      <c r="E5" s="222"/>
+      <c r="F5" s="222"/>
+      <c r="G5" s="222"/>
+      <c r="H5" s="222"/>
+      <c r="I5" s="222"/>
+      <c r="J5" s="222"/>
+      <c r="K5" s="222"/>
+      <c r="L5" s="222"/>
       <c r="P5" s="228"/>
       <c r="Q5" s="228"/>
       <c r="R5" s="228"/>
@@ -6732,18 +6697,18 @@
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B11" s="145"/>
-      <c r="C11" s="219" t="s">
+      <c r="C11" s="222" t="s">
         <v>301</v>
       </c>
-      <c r="D11" s="219"/>
-      <c r="E11" s="219"/>
-      <c r="F11" s="219"/>
-      <c r="G11" s="219"/>
-      <c r="H11" s="219"/>
-      <c r="I11" s="219"/>
-      <c r="J11" s="219"/>
-      <c r="K11" s="219"/>
-      <c r="L11" s="219"/>
+      <c r="D11" s="222"/>
+      <c r="E11" s="222"/>
+      <c r="F11" s="222"/>
+      <c r="G11" s="222"/>
+      <c r="H11" s="222"/>
+      <c r="I11" s="222"/>
+      <c r="J11" s="222"/>
+      <c r="K11" s="222"/>
+      <c r="L11" s="222"/>
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B12" s="7" t="s">
@@ -7013,18 +6978,18 @@
       <c r="C19" s="162"/>
     </row>
     <row r="21" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="C21" s="219" t="s">
+      <c r="C21" s="222" t="s">
         <v>309</v>
       </c>
-      <c r="D21" s="219"/>
-      <c r="E21" s="219"/>
-      <c r="F21" s="219"/>
-      <c r="G21" s="219"/>
-      <c r="H21" s="219"/>
-      <c r="I21" s="219"/>
-      <c r="J21" s="219"/>
-      <c r="K21" s="219"/>
-      <c r="L21" s="219"/>
+      <c r="D21" s="222"/>
+      <c r="E21" s="222"/>
+      <c r="F21" s="222"/>
+      <c r="G21" s="222"/>
+      <c r="H21" s="222"/>
+      <c r="I21" s="222"/>
+      <c r="J21" s="222"/>
+      <c r="K21" s="222"/>
+      <c r="L21" s="222"/>
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B22" s="7" t="s">
@@ -7247,10 +7212,10 @@
       </c>
     </row>
     <row r="29" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B29" s="220" t="s">
+      <c r="B29" s="223" t="s">
         <v>305</v>
       </c>
-      <c r="C29" s="220"/>
+      <c r="C29" s="223"/>
     </row>
     <row r="30" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B30" s="1" t="s">
@@ -7278,18 +7243,18 @@
     </row>
     <row r="35" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B35" s="92"/>
-      <c r="C35" s="219" t="s">
+      <c r="C35" s="222" t="s">
         <v>178</v>
       </c>
-      <c r="D35" s="219"/>
-      <c r="E35" s="219"/>
-      <c r="F35" s="219"/>
-      <c r="G35" s="219"/>
-      <c r="H35" s="219"/>
-      <c r="I35" s="219"/>
-      <c r="J35" s="219"/>
-      <c r="K35" s="219"/>
-      <c r="L35" s="219"/>
+      <c r="D35" s="222"/>
+      <c r="E35" s="222"/>
+      <c r="F35" s="222"/>
+      <c r="G35" s="222"/>
+      <c r="H35" s="222"/>
+      <c r="I35" s="222"/>
+      <c r="J35" s="222"/>
+      <c r="K35" s="222"/>
+      <c r="L35" s="222"/>
     </row>
     <row r="36" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B36" s="7" t="s">
@@ -7382,18 +7347,18 @@
       </c>
     </row>
     <row r="39" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="C39" s="219" t="s">
+      <c r="C39" s="222" t="s">
         <v>317</v>
       </c>
-      <c r="D39" s="219"/>
-      <c r="E39" s="219"/>
-      <c r="F39" s="219"/>
-      <c r="G39" s="219"/>
-      <c r="H39" s="219"/>
-      <c r="I39" s="219"/>
-      <c r="J39" s="219"/>
-      <c r="K39" s="219"/>
-      <c r="L39" s="219"/>
+      <c r="D39" s="222"/>
+      <c r="E39" s="222"/>
+      <c r="F39" s="222"/>
+      <c r="G39" s="222"/>
+      <c r="H39" s="222"/>
+      <c r="I39" s="222"/>
+      <c r="J39" s="222"/>
+      <c r="K39" s="222"/>
+      <c r="L39" s="222"/>
     </row>
     <row r="40" spans="2:12" x14ac:dyDescent="0.2">
       <c r="C40" s="180">
@@ -7528,18 +7493,18 @@
       </c>
     </row>
     <row r="44" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="C44" s="219" t="s">
+      <c r="C44" s="222" t="s">
         <v>319</v>
       </c>
-      <c r="D44" s="219"/>
-      <c r="E44" s="219"/>
-      <c r="F44" s="219"/>
-      <c r="G44" s="219"/>
-      <c r="H44" s="219"/>
-      <c r="I44" s="219"/>
-      <c r="J44" s="219"/>
-      <c r="K44" s="219"/>
-      <c r="L44" s="219"/>
+      <c r="D44" s="222"/>
+      <c r="E44" s="222"/>
+      <c r="F44" s="222"/>
+      <c r="G44" s="222"/>
+      <c r="H44" s="222"/>
+      <c r="I44" s="222"/>
+      <c r="J44" s="222"/>
+      <c r="K44" s="222"/>
+      <c r="L44" s="222"/>
     </row>
     <row r="45" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B45" s="7" t="s">
@@ -7737,20 +7702,20 @@
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A2" s="103"/>
-      <c r="C2" s="220" t="s">
+      <c r="C2" s="223" t="s">
         <v>168</v>
       </c>
-      <c r="D2" s="220"/>
-      <c r="E2" s="220"/>
-      <c r="F2" s="220"/>
-      <c r="G2" s="223"/>
-      <c r="H2" s="224" t="s">
+      <c r="D2" s="223"/>
+      <c r="E2" s="223"/>
+      <c r="F2" s="223"/>
+      <c r="G2" s="226"/>
+      <c r="H2" s="227" t="s">
         <v>169</v>
       </c>
-      <c r="I2" s="220"/>
-      <c r="J2" s="220"/>
-      <c r="K2" s="220"/>
-      <c r="L2" s="220"/>
+      <c r="I2" s="223"/>
+      <c r="J2" s="223"/>
+      <c r="K2" s="223"/>
+      <c r="L2" s="223"/>
       <c r="S2" s="228"/>
       <c r="T2" s="228"/>
       <c r="U2" s="228"/>
@@ -7768,18 +7733,18 @@
     <row r="4" spans="1:31" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="108"/>
       <c r="B4" s="92"/>
-      <c r="C4" s="219" t="s">
+      <c r="C4" s="222" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="219"/>
-      <c r="E4" s="219"/>
-      <c r="F4" s="219"/>
-      <c r="G4" s="219"/>
-      <c r="H4" s="219"/>
-      <c r="I4" s="219"/>
-      <c r="J4" s="219"/>
-      <c r="K4" s="219"/>
-      <c r="L4" s="219"/>
+      <c r="D4" s="222"/>
+      <c r="E4" s="222"/>
+      <c r="F4" s="222"/>
+      <c r="G4" s="222"/>
+      <c r="H4" s="222"/>
+      <c r="I4" s="222"/>
+      <c r="J4" s="222"/>
+      <c r="K4" s="222"/>
+      <c r="L4" s="222"/>
       <c r="S4" s="228"/>
       <c r="T4" s="228"/>
       <c r="U4" s="228"/>
@@ -8574,18 +8539,18 @@
       <c r="AE17" s="112"/>
     </row>
     <row r="20" spans="2:31" x14ac:dyDescent="0.2">
-      <c r="C20" s="219" t="s">
+      <c r="C20" s="222" t="s">
         <v>275</v>
       </c>
-      <c r="D20" s="219"/>
-      <c r="E20" s="219"/>
-      <c r="F20" s="219"/>
-      <c r="G20" s="219"/>
-      <c r="H20" s="219"/>
-      <c r="I20" s="219"/>
-      <c r="J20" s="219"/>
-      <c r="K20" s="219"/>
-      <c r="L20" s="219"/>
+      <c r="D20" s="222"/>
+      <c r="E20" s="222"/>
+      <c r="F20" s="222"/>
+      <c r="G20" s="222"/>
+      <c r="H20" s="222"/>
+      <c r="I20" s="222"/>
+      <c r="J20" s="222"/>
+      <c r="K20" s="222"/>
+      <c r="L20" s="222"/>
     </row>
     <row r="21" spans="2:31" x14ac:dyDescent="0.2">
       <c r="C21" s="62">
@@ -8717,20 +8682,20 @@
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A2" s="103"/>
-      <c r="C2" s="220" t="s">
+      <c r="C2" s="223" t="s">
         <v>168</v>
       </c>
-      <c r="D2" s="220"/>
-      <c r="E2" s="220"/>
-      <c r="F2" s="220"/>
-      <c r="G2" s="223"/>
-      <c r="H2" s="224" t="s">
+      <c r="D2" s="223"/>
+      <c r="E2" s="223"/>
+      <c r="F2" s="223"/>
+      <c r="G2" s="226"/>
+      <c r="H2" s="227" t="s">
         <v>169</v>
       </c>
-      <c r="I2" s="220"/>
-      <c r="J2" s="220"/>
-      <c r="K2" s="220"/>
-      <c r="L2" s="220"/>
+      <c r="I2" s="223"/>
+      <c r="J2" s="223"/>
+      <c r="K2" s="223"/>
+      <c r="L2" s="223"/>
       <c r="S2" s="228"/>
       <c r="T2" s="228"/>
       <c r="U2" s="228"/>
@@ -8748,18 +8713,18 @@
     <row r="4" spans="1:31" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="108"/>
       <c r="B4" s="92"/>
-      <c r="C4" s="219" t="s">
+      <c r="C4" s="222" t="s">
         <v>257</v>
       </c>
-      <c r="D4" s="219"/>
-      <c r="E4" s="219"/>
-      <c r="F4" s="219"/>
-      <c r="G4" s="219"/>
-      <c r="H4" s="219"/>
-      <c r="I4" s="219"/>
-      <c r="J4" s="219"/>
-      <c r="K4" s="219"/>
-      <c r="L4" s="219"/>
+      <c r="D4" s="222"/>
+      <c r="E4" s="222"/>
+      <c r="F4" s="222"/>
+      <c r="G4" s="222"/>
+      <c r="H4" s="222"/>
+      <c r="I4" s="222"/>
+      <c r="J4" s="222"/>
+      <c r="K4" s="222"/>
+      <c r="L4" s="222"/>
       <c r="S4" s="228"/>
       <c r="T4" s="228"/>
       <c r="U4" s="228"/>
@@ -10507,20 +10472,20 @@
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A2" s="103"/>
-      <c r="C2" s="220" t="s">
+      <c r="C2" s="223" t="s">
         <v>168</v>
       </c>
-      <c r="D2" s="220"/>
-      <c r="E2" s="220"/>
-      <c r="F2" s="220"/>
-      <c r="G2" s="223"/>
-      <c r="H2" s="224" t="s">
+      <c r="D2" s="223"/>
+      <c r="E2" s="223"/>
+      <c r="F2" s="223"/>
+      <c r="G2" s="226"/>
+      <c r="H2" s="227" t="s">
         <v>169</v>
       </c>
-      <c r="I2" s="220"/>
-      <c r="J2" s="220"/>
-      <c r="K2" s="220"/>
-      <c r="L2" s="220"/>
+      <c r="I2" s="223"/>
+      <c r="J2" s="223"/>
+      <c r="K2" s="223"/>
+      <c r="L2" s="223"/>
       <c r="S2" s="228"/>
       <c r="T2" s="228"/>
       <c r="U2" s="228"/>
@@ -10538,18 +10503,18 @@
     <row r="4" spans="1:31" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="108"/>
       <c r="B4" s="92"/>
-      <c r="C4" s="219" t="s">
+      <c r="C4" s="222" t="s">
         <v>258</v>
       </c>
-      <c r="D4" s="219"/>
-      <c r="E4" s="219"/>
-      <c r="F4" s="219"/>
-      <c r="G4" s="219"/>
-      <c r="H4" s="219"/>
-      <c r="I4" s="219"/>
-      <c r="J4" s="219"/>
-      <c r="K4" s="219"/>
-      <c r="L4" s="219"/>
+      <c r="D4" s="222"/>
+      <c r="E4" s="222"/>
+      <c r="F4" s="222"/>
+      <c r="G4" s="222"/>
+      <c r="H4" s="222"/>
+      <c r="I4" s="222"/>
+      <c r="J4" s="222"/>
+      <c r="K4" s="222"/>
+      <c r="L4" s="222"/>
       <c r="S4" s="228"/>
       <c r="T4" s="228"/>
       <c r="U4" s="228"/>
@@ -11828,18 +11793,18 @@
       <c r="I27" s="107"/>
     </row>
     <row r="29" spans="2:31" x14ac:dyDescent="0.2">
-      <c r="C29" s="219" t="s">
+      <c r="C29" s="222" t="s">
         <v>275</v>
       </c>
-      <c r="D29" s="219"/>
-      <c r="E29" s="219"/>
-      <c r="F29" s="219"/>
-      <c r="G29" s="219"/>
-      <c r="H29" s="219"/>
-      <c r="I29" s="219"/>
-      <c r="J29" s="219"/>
-      <c r="K29" s="219"/>
-      <c r="L29" s="219"/>
+      <c r="D29" s="222"/>
+      <c r="E29" s="222"/>
+      <c r="F29" s="222"/>
+      <c r="G29" s="222"/>
+      <c r="H29" s="222"/>
+      <c r="I29" s="222"/>
+      <c r="J29" s="222"/>
+      <c r="K29" s="222"/>
+      <c r="L29" s="222"/>
     </row>
     <row r="30" spans="2:31" x14ac:dyDescent="0.2">
       <c r="C30" s="62">
@@ -12190,10 +12155,10 @@
     </row>
     <row r="3" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="220" t="s">
+      <c r="B4" s="223" t="s">
         <v>340</v>
       </c>
-      <c r="C4" s="220"/>
+      <c r="C4" s="223"/>
     </row>
     <row r="5" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="1" t="s">
@@ -12273,10 +12238,10 @@
     </row>
     <row r="14" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="15" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="220" t="s">
+      <c r="B15" s="223" t="s">
         <v>346</v>
       </c>
-      <c r="C15" s="220"/>
+      <c r="C15" s="223"/>
     </row>
     <row r="16" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="1" t="s">
@@ -12388,20 +12353,20 @@
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A3" s="103"/>
-      <c r="C3" s="220" t="s">
+      <c r="C3" s="223" t="s">
         <v>168</v>
       </c>
-      <c r="D3" s="220"/>
-      <c r="E3" s="220"/>
-      <c r="F3" s="220"/>
-      <c r="G3" s="223"/>
-      <c r="H3" s="224" t="s">
+      <c r="D3" s="223"/>
+      <c r="E3" s="223"/>
+      <c r="F3" s="223"/>
+      <c r="G3" s="226"/>
+      <c r="H3" s="227" t="s">
         <v>169</v>
       </c>
-      <c r="I3" s="220"/>
-      <c r="J3" s="220"/>
-      <c r="K3" s="220"/>
-      <c r="L3" s="220"/>
+      <c r="I3" s="223"/>
+      <c r="J3" s="223"/>
+      <c r="K3" s="223"/>
+      <c r="L3" s="223"/>
       <c r="P3" s="228"/>
       <c r="Q3" s="228"/>
       <c r="R3" s="228"/>
@@ -12419,18 +12384,18 @@
     <row r="5" spans="1:28" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="108"/>
       <c r="B5" s="92"/>
-      <c r="C5" s="219" t="s">
+      <c r="C5" s="222" t="s">
         <v>360</v>
       </c>
-      <c r="D5" s="219"/>
-      <c r="E5" s="219"/>
-      <c r="F5" s="219"/>
-      <c r="G5" s="219"/>
-      <c r="H5" s="219"/>
-      <c r="I5" s="219"/>
-      <c r="J5" s="219"/>
-      <c r="K5" s="219"/>
-      <c r="L5" s="219"/>
+      <c r="D5" s="222"/>
+      <c r="E5" s="222"/>
+      <c r="F5" s="222"/>
+      <c r="G5" s="222"/>
+      <c r="H5" s="222"/>
+      <c r="I5" s="222"/>
+      <c r="J5" s="222"/>
+      <c r="K5" s="222"/>
+      <c r="L5" s="222"/>
       <c r="P5" s="228"/>
       <c r="Q5" s="228"/>
       <c r="R5" s="228"/>
@@ -12687,10 +12652,10 @@
       </c>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="B13" s="220" t="s">
+      <c r="B13" s="223" t="s">
         <v>361</v>
       </c>
-      <c r="C13" s="220"/>
+      <c r="C13" s="223"/>
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B14" s="1" t="s">
@@ -12710,10 +12675,10 @@
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B18" s="220" t="s">
+      <c r="B18" s="223" t="s">
         <v>91</v>
       </c>
-      <c r="C18" s="220"/>
+      <c r="C18" s="223"/>
     </row>
     <row r="19" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B19" s="1" t="s">
@@ -12827,37 +12792,37 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="103"/>
-      <c r="C2" s="220" t="s">
+      <c r="C2" s="223" t="s">
         <v>168</v>
       </c>
-      <c r="D2" s="220"/>
-      <c r="E2" s="220"/>
-      <c r="F2" s="220"/>
-      <c r="G2" s="223"/>
-      <c r="H2" s="224" t="s">
+      <c r="D2" s="223"/>
+      <c r="E2" s="223"/>
+      <c r="F2" s="223"/>
+      <c r="G2" s="226"/>
+      <c r="H2" s="227" t="s">
         <v>169</v>
       </c>
-      <c r="I2" s="220"/>
-      <c r="J2" s="220"/>
-      <c r="K2" s="220"/>
-      <c r="L2" s="220"/>
+      <c r="I2" s="223"/>
+      <c r="J2" s="223"/>
+      <c r="K2" s="223"/>
+      <c r="L2" s="223"/>
     </row>
     <row r="3" spans="1:14" ht="10" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="1:14" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="108"/>
       <c r="B4" s="92"/>
-      <c r="C4" s="219" t="s">
+      <c r="C4" s="222" t="s">
         <v>178</v>
       </c>
-      <c r="D4" s="219"/>
-      <c r="E4" s="219"/>
-      <c r="F4" s="219"/>
-      <c r="G4" s="219"/>
-      <c r="H4" s="219"/>
-      <c r="I4" s="219"/>
-      <c r="J4" s="219"/>
-      <c r="K4" s="219"/>
-      <c r="L4" s="219"/>
+      <c r="D4" s="222"/>
+      <c r="E4" s="222"/>
+      <c r="F4" s="222"/>
+      <c r="G4" s="222"/>
+      <c r="H4" s="222"/>
+      <c r="I4" s="222"/>
+      <c r="J4" s="222"/>
+      <c r="K4" s="222"/>
+      <c r="L4" s="222"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B5" s="7" t="s">
@@ -13000,18 +12965,18 @@
       <c r="N8" s="91"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="C9" s="219" t="s">
+      <c r="C9" s="222" t="s">
         <v>184</v>
       </c>
-      <c r="D9" s="219"/>
-      <c r="E9" s="219"/>
-      <c r="F9" s="219"/>
-      <c r="G9" s="219"/>
-      <c r="H9" s="219"/>
-      <c r="I9" s="219"/>
-      <c r="J9" s="219"/>
-      <c r="K9" s="219"/>
-      <c r="L9" s="219"/>
+      <c r="D9" s="222"/>
+      <c r="E9" s="222"/>
+      <c r="F9" s="222"/>
+      <c r="G9" s="222"/>
+      <c r="H9" s="222"/>
+      <c r="I9" s="222"/>
+      <c r="J9" s="222"/>
+      <c r="K9" s="222"/>
+      <c r="L9" s="222"/>
       <c r="N9" s="91"/>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
@@ -13162,18 +13127,18 @@
       <c r="N13" s="91"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="C14" s="219" t="s">
+      <c r="C14" s="222" t="s">
         <v>409</v>
       </c>
-      <c r="D14" s="219"/>
-      <c r="E14" s="219"/>
-      <c r="F14" s="219"/>
-      <c r="G14" s="219"/>
-      <c r="H14" s="219"/>
-      <c r="I14" s="219"/>
-      <c r="J14" s="219"/>
-      <c r="K14" s="219"/>
-      <c r="L14" s="219"/>
+      <c r="D14" s="222"/>
+      <c r="E14" s="222"/>
+      <c r="F14" s="222"/>
+      <c r="G14" s="222"/>
+      <c r="H14" s="222"/>
+      <c r="I14" s="222"/>
+      <c r="J14" s="222"/>
+      <c r="K14" s="222"/>
+      <c r="L14" s="222"/>
       <c r="N14" s="91"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.2">
@@ -13310,10 +13275,10 @@
       <c r="N19" s="91"/>
     </row>
     <row r="20" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B20" s="220" t="s">
+      <c r="B20" s="223" t="s">
         <v>377</v>
       </c>
-      <c r="C20" s="220"/>
+      <c r="C20" s="223"/>
       <c r="N20" s="91"/>
     </row>
     <row r="21" spans="2:14" x14ac:dyDescent="0.2">
@@ -13370,10 +13335,10 @@
       </c>
     </row>
     <row r="28" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B28" s="220" t="s">
+      <c r="B28" s="223" t="s">
         <v>380</v>
       </c>
-      <c r="C28" s="220"/>
+      <c r="C28" s="223"/>
     </row>
     <row r="29" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B29" s="1" t="s">
@@ -13471,10 +13436,10 @@
       <c r="N3" s="91"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B4" s="220" t="s">
+      <c r="B4" s="223" t="s">
         <v>390</v>
       </c>
-      <c r="C4" s="220"/>
+      <c r="C4" s="223"/>
       <c r="N4" s="91"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
@@ -16635,11 +16600,11 @@
         <v>86</v>
       </c>
       <c r="O4" s="4"/>
-      <c r="P4" s="225" t="s">
+      <c r="P4" s="219" t="s">
         <v>87</v>
       </c>
-      <c r="Q4" s="226"/>
-      <c r="R4" s="227"/>
+      <c r="Q4" s="220"/>
+      <c r="R4" s="221"/>
       <c r="S4" s="4"/>
     </row>
     <row r="5" spans="1:19" s="18" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.2">
@@ -19815,7 +19780,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8047DB4-BCDE-EC47-A3C5-C98010D5458E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8047DB4-BCDE-EC47-A3C5-C98010D5458E}">
   <dimension ref="B2:S96"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" outlineLevelRow="1" x14ac:dyDescent="0.2"/>
   <cols>
@@ -20100,7 +20065,7 @@
         <v>0</v>
       </c>
       <c r="S6" s="164">
-        <f t="shared" ref="S6:S20" si="0">SUM(N6:Q6)</f>
+        <f t="shared" ref="S6:S18" si="0">SUM(N6:Q6)</f>
         <v>0</v>
       </c>
     </row>
@@ -20844,7 +20809,8 @@
         <v>0</v>
       </c>
       <c r="H18" s="195">
-        <v>166870</v>
+        <f>'Statement Y'!H18</f>
+        <v>0</v>
       </c>
       <c r="J18" s="195">
         <f>'Statement Q'!C18</f>
@@ -20871,7 +20837,8 @@
         <v>0</v>
       </c>
       <c r="P18" s="195">
-        <v>45000</v>
+        <f>'Statement Q'!I18</f>
+        <v>0</v>
       </c>
       <c r="Q18" s="195">
         <f>'Statement Q'!J18</f>
@@ -20879,7 +20846,7 @@
       </c>
       <c r="S18" s="195">
         <f t="shared" si="0"/>
-        <v>45000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="2:19" outlineLevel="1" x14ac:dyDescent="0.2">
@@ -20971,9 +20938,9 @@
         <f>'Statement Y'!G22</f>
         <v>0</v>
       </c>
-      <c r="H20" s="196" t="e">
-        <f>H18/H19</f>
-        <v>#DIV/0!</v>
+      <c r="H20" s="196">
+        <f>'Statement Y'!H22</f>
+        <v>0</v>
       </c>
       <c r="J20" s="197">
         <f>'Statement Q'!C22</f>
@@ -20999,16 +20966,16 @@
         <f>'Statement Q'!H22</f>
         <v>0</v>
       </c>
-      <c r="P20" s="197" t="e">
-        <f>P18/P19</f>
-        <v>#DIV/0!</v>
+      <c r="P20" s="197">
+        <f>'Statement Q'!I22</f>
+        <v>0</v>
       </c>
       <c r="Q20" s="197">
         <f>'Statement Q'!J22</f>
         <v>0</v>
       </c>
       <c r="S20" s="197" t="e">
-        <f t="shared" si="0"/>
+        <f>S18/S19</f>
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -24875,7 +24842,7 @@
       </c>
       <c r="H89" s="203">
         <f t="shared" si="24"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J89" s="205"/>
       <c r="K89" s="203">
@@ -24903,11 +24870,11 @@
       </c>
       <c r="P89" s="203">
         <f t="shared" si="25"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q89" s="203">
         <f t="shared" si="25"/>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="S89" s="205"/>
     </row>
@@ -24994,9 +24961,9 @@
         <f t="shared" si="28"/>
         <v>0</v>
       </c>
-      <c r="H91" s="201" t="e">
+      <c r="H91" s="201">
         <f t="shared" si="28"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="J91" s="205"/>
       <c r="K91" s="201">
@@ -25022,13 +24989,13 @@
         <f t="shared" si="29"/>
         <v>0</v>
       </c>
-      <c r="P91" s="201" t="e">
+      <c r="P91" s="201">
         <f t="shared" si="29"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q91" s="201" t="e">
+        <v>0</v>
+      </c>
+      <c r="Q91" s="201">
         <f t="shared" si="29"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="S91" s="205"/>
     </row>
@@ -25253,7 +25220,6 @@
     <ignoredError sqref="S19 C79:H79 S79 D90:H90 K90:Q90" formula="1"/>
     <ignoredError sqref="C63:H63 J63:Q63 S69" formulaRange="1"/>
   </ignoredErrors>
-  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -25310,36 +25276,36 @@
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A2" s="103"/>
-      <c r="C2" s="220" t="s">
+      <c r="C2" s="223" t="s">
         <v>168</v>
       </c>
-      <c r="D2" s="220"/>
-      <c r="E2" s="220"/>
-      <c r="F2" s="220"/>
-      <c r="G2" s="223"/>
-      <c r="H2" s="224" t="s">
+      <c r="D2" s="223"/>
+      <c r="E2" s="223"/>
+      <c r="F2" s="223"/>
+      <c r="G2" s="226"/>
+      <c r="H2" s="227" t="s">
         <v>169</v>
       </c>
-      <c r="I2" s="220"/>
-      <c r="J2" s="220"/>
-      <c r="K2" s="220"/>
-      <c r="L2" s="220"/>
+      <c r="I2" s="223"/>
+      <c r="J2" s="223"/>
+      <c r="K2" s="223"/>
+      <c r="L2" s="223"/>
       <c r="O2" s="90"/>
-      <c r="S2" s="220" t="s">
+      <c r="S2" s="223" t="s">
         <v>168</v>
       </c>
-      <c r="T2" s="220"/>
-      <c r="U2" s="220"/>
-      <c r="V2" s="220"/>
-      <c r="W2" s="220"/>
-      <c r="X2" s="220"/>
-      <c r="Y2" s="220"/>
-      <c r="Z2" s="220"/>
-      <c r="AA2" s="220" t="s">
+      <c r="T2" s="223"/>
+      <c r="U2" s="223"/>
+      <c r="V2" s="223"/>
+      <c r="W2" s="223"/>
+      <c r="X2" s="223"/>
+      <c r="Y2" s="223"/>
+      <c r="Z2" s="223"/>
+      <c r="AA2" s="223" t="s">
         <v>169</v>
       </c>
-      <c r="AB2" s="220"/>
-      <c r="AC2" s="220"/>
+      <c r="AB2" s="223"/>
+      <c r="AC2" s="223"/>
       <c r="AE2" s="127" t="s">
         <v>86</v>
       </c>
@@ -25350,32 +25316,32 @@
     <row r="4" spans="1:31" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="108"/>
       <c r="B4" s="92"/>
-      <c r="C4" s="219" t="s">
+      <c r="C4" s="222" t="s">
         <v>178</v>
       </c>
-      <c r="D4" s="219"/>
-      <c r="E4" s="219"/>
-      <c r="F4" s="219"/>
-      <c r="G4" s="219"/>
-      <c r="H4" s="219"/>
-      <c r="I4" s="219"/>
-      <c r="J4" s="219"/>
-      <c r="K4" s="219"/>
-      <c r="L4" s="219"/>
+      <c r="D4" s="222"/>
+      <c r="E4" s="222"/>
+      <c r="F4" s="222"/>
+      <c r="G4" s="222"/>
+      <c r="H4" s="222"/>
+      <c r="I4" s="222"/>
+      <c r="J4" s="222"/>
+      <c r="K4" s="222"/>
+      <c r="L4" s="222"/>
       <c r="O4" s="90"/>
-      <c r="S4" s="221" t="s">
+      <c r="S4" s="224" t="s">
         <v>178</v>
       </c>
-      <c r="T4" s="222"/>
-      <c r="U4" s="222"/>
-      <c r="V4" s="222"/>
-      <c r="W4" s="222"/>
-      <c r="X4" s="222"/>
-      <c r="Y4" s="222"/>
-      <c r="Z4" s="222"/>
-      <c r="AA4" s="222"/>
-      <c r="AB4" s="222"/>
-      <c r="AC4" s="222"/>
+      <c r="T4" s="225"/>
+      <c r="U4" s="225"/>
+      <c r="V4" s="225"/>
+      <c r="W4" s="225"/>
+      <c r="X4" s="225"/>
+      <c r="Y4" s="225"/>
+      <c r="Z4" s="225"/>
+      <c r="AA4" s="225"/>
+      <c r="AB4" s="225"/>
+      <c r="AC4" s="225"/>
       <c r="AE4" s="138" t="s">
         <v>202</v>
       </c>
@@ -26171,33 +26137,33 @@
       <c r="Q13" s="91"/>
     </row>
     <row r="14" spans="1:31" x14ac:dyDescent="0.2">
-      <c r="C14" s="219" t="s">
+      <c r="C14" s="222" t="s">
         <v>184</v>
       </c>
-      <c r="D14" s="219"/>
-      <c r="E14" s="219"/>
-      <c r="F14" s="219"/>
-      <c r="G14" s="219"/>
-      <c r="H14" s="219"/>
-      <c r="I14" s="219"/>
-      <c r="J14" s="219"/>
-      <c r="K14" s="219"/>
-      <c r="L14" s="219"/>
+      <c r="D14" s="222"/>
+      <c r="E14" s="222"/>
+      <c r="F14" s="222"/>
+      <c r="G14" s="222"/>
+      <c r="H14" s="222"/>
+      <c r="I14" s="222"/>
+      <c r="J14" s="222"/>
+      <c r="K14" s="222"/>
+      <c r="L14" s="222"/>
       <c r="O14" s="90"/>
       <c r="Q14" s="91"/>
-      <c r="S14" s="221" t="s">
+      <c r="S14" s="224" t="s">
         <v>184</v>
       </c>
-      <c r="T14" s="222"/>
-      <c r="U14" s="222"/>
-      <c r="V14" s="222"/>
-      <c r="W14" s="222"/>
-      <c r="X14" s="222"/>
-      <c r="Y14" s="222"/>
-      <c r="Z14" s="222"/>
-      <c r="AA14" s="222"/>
-      <c r="AB14" s="222"/>
-      <c r="AC14" s="222"/>
+      <c r="T14" s="225"/>
+      <c r="U14" s="225"/>
+      <c r="V14" s="225"/>
+      <c r="W14" s="225"/>
+      <c r="X14" s="225"/>
+      <c r="Y14" s="225"/>
+      <c r="Z14" s="225"/>
+      <c r="AA14" s="225"/>
+      <c r="AB14" s="225"/>
+      <c r="AC14" s="225"/>
     </row>
     <row r="15" spans="1:31" x14ac:dyDescent="0.2">
       <c r="B15" s="7" t="s">
@@ -26890,33 +26856,33 @@
       <c r="Q24" s="91"/>
     </row>
     <row r="25" spans="2:31" x14ac:dyDescent="0.2">
-      <c r="C25" s="219" t="s">
+      <c r="C25" s="222" t="s">
         <v>186</v>
       </c>
-      <c r="D25" s="219"/>
-      <c r="E25" s="219"/>
-      <c r="F25" s="219"/>
-      <c r="G25" s="219"/>
-      <c r="H25" s="219"/>
-      <c r="I25" s="219"/>
-      <c r="J25" s="219"/>
-      <c r="K25" s="219"/>
-      <c r="L25" s="219"/>
+      <c r="D25" s="222"/>
+      <c r="E25" s="222"/>
+      <c r="F25" s="222"/>
+      <c r="G25" s="222"/>
+      <c r="H25" s="222"/>
+      <c r="I25" s="222"/>
+      <c r="J25" s="222"/>
+      <c r="K25" s="222"/>
+      <c r="L25" s="222"/>
       <c r="O25" s="90"/>
       <c r="Q25" s="91"/>
-      <c r="S25" s="221" t="s">
+      <c r="S25" s="224" t="s">
         <v>186</v>
       </c>
-      <c r="T25" s="222"/>
-      <c r="U25" s="222"/>
-      <c r="V25" s="222"/>
-      <c r="W25" s="222"/>
-      <c r="X25" s="222"/>
-      <c r="Y25" s="222"/>
-      <c r="Z25" s="222"/>
-      <c r="AA25" s="222"/>
-      <c r="AB25" s="222"/>
-      <c r="AC25" s="222"/>
+      <c r="T25" s="225"/>
+      <c r="U25" s="225"/>
+      <c r="V25" s="225"/>
+      <c r="W25" s="225"/>
+      <c r="X25" s="225"/>
+      <c r="Y25" s="225"/>
+      <c r="Z25" s="225"/>
+      <c r="AA25" s="225"/>
+      <c r="AB25" s="225"/>
+      <c r="AC25" s="225"/>
       <c r="AE25" s="138" t="str">
         <f>AE4</f>
         <v>Q1-Q2-Q3</v>
@@ -28239,32 +28205,32 @@
       <c r="O42" s="90"/>
     </row>
     <row r="43" spans="2:31" x14ac:dyDescent="0.2">
-      <c r="C43" s="219" t="s">
+      <c r="C43" s="222" t="s">
         <v>197</v>
       </c>
-      <c r="D43" s="219"/>
-      <c r="E43" s="219"/>
-      <c r="F43" s="219"/>
-      <c r="G43" s="219"/>
-      <c r="H43" s="219"/>
-      <c r="I43" s="219"/>
-      <c r="J43" s="219"/>
-      <c r="K43" s="219"/>
-      <c r="L43" s="219"/>
+      <c r="D43" s="222"/>
+      <c r="E43" s="222"/>
+      <c r="F43" s="222"/>
+      <c r="G43" s="222"/>
+      <c r="H43" s="222"/>
+      <c r="I43" s="222"/>
+      <c r="J43" s="222"/>
+      <c r="K43" s="222"/>
+      <c r="L43" s="222"/>
       <c r="O43" s="90"/>
-      <c r="S43" s="221" t="s">
+      <c r="S43" s="224" t="s">
         <v>197</v>
       </c>
-      <c r="T43" s="222"/>
-      <c r="U43" s="222"/>
-      <c r="V43" s="222"/>
-      <c r="W43" s="222"/>
-      <c r="X43" s="222"/>
-      <c r="Y43" s="222"/>
-      <c r="Z43" s="222"/>
-      <c r="AA43" s="222"/>
-      <c r="AB43" s="222"/>
-      <c r="AC43" s="222"/>
+      <c r="T43" s="225"/>
+      <c r="U43" s="225"/>
+      <c r="V43" s="225"/>
+      <c r="W43" s="225"/>
+      <c r="X43" s="225"/>
+      <c r="Y43" s="225"/>
+      <c r="Z43" s="225"/>
+      <c r="AA43" s="225"/>
+      <c r="AB43" s="225"/>
+      <c r="AC43" s="225"/>
     </row>
     <row r="44" spans="2:31" x14ac:dyDescent="0.2">
       <c r="B44" s="7" t="s">
@@ -28880,35 +28846,35 @@
     </row>
     <row r="2" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A2" s="103"/>
-      <c r="C2" s="220" t="s">
+      <c r="C2" s="223" t="s">
         <v>168</v>
       </c>
-      <c r="D2" s="220"/>
-      <c r="E2" s="220"/>
-      <c r="F2" s="220"/>
-      <c r="G2" s="223"/>
-      <c r="H2" s="224" t="s">
+      <c r="D2" s="223"/>
+      <c r="E2" s="223"/>
+      <c r="F2" s="223"/>
+      <c r="G2" s="226"/>
+      <c r="H2" s="227" t="s">
         <v>169</v>
       </c>
-      <c r="I2" s="220"/>
-      <c r="J2" s="220"/>
-      <c r="K2" s="220"/>
-      <c r="L2" s="220"/>
-      <c r="P2" s="220" t="s">
+      <c r="I2" s="223"/>
+      <c r="J2" s="223"/>
+      <c r="K2" s="223"/>
+      <c r="L2" s="223"/>
+      <c r="P2" s="223" t="s">
         <v>168</v>
       </c>
-      <c r="Q2" s="220"/>
-      <c r="R2" s="220"/>
-      <c r="S2" s="220"/>
-      <c r="T2" s="220"/>
-      <c r="U2" s="220"/>
-      <c r="V2" s="220"/>
-      <c r="W2" s="220"/>
-      <c r="X2" s="220" t="s">
+      <c r="Q2" s="223"/>
+      <c r="R2" s="223"/>
+      <c r="S2" s="223"/>
+      <c r="T2" s="223"/>
+      <c r="U2" s="223"/>
+      <c r="V2" s="223"/>
+      <c r="W2" s="223"/>
+      <c r="X2" s="223" t="s">
         <v>169</v>
       </c>
-      <c r="Y2" s="220"/>
-      <c r="Z2" s="220"/>
+      <c r="Y2" s="223"/>
+      <c r="Z2" s="223"/>
       <c r="AB2" s="127" t="s">
         <v>86</v>
       </c>
@@ -28917,31 +28883,31 @@
     <row r="4" spans="1:28" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="108"/>
       <c r="B4" s="92"/>
-      <c r="C4" s="219" t="s">
+      <c r="C4" s="222" t="s">
         <v>178</v>
       </c>
-      <c r="D4" s="219"/>
-      <c r="E4" s="219"/>
-      <c r="F4" s="219"/>
-      <c r="G4" s="219"/>
-      <c r="H4" s="219"/>
-      <c r="I4" s="219"/>
-      <c r="J4" s="219"/>
-      <c r="K4" s="219"/>
-      <c r="L4" s="219"/>
-      <c r="P4" s="222" t="s">
+      <c r="D4" s="222"/>
+      <c r="E4" s="222"/>
+      <c r="F4" s="222"/>
+      <c r="G4" s="222"/>
+      <c r="H4" s="222"/>
+      <c r="I4" s="222"/>
+      <c r="J4" s="222"/>
+      <c r="K4" s="222"/>
+      <c r="L4" s="222"/>
+      <c r="P4" s="225" t="s">
         <v>178</v>
       </c>
-      <c r="Q4" s="222"/>
-      <c r="R4" s="222"/>
-      <c r="S4" s="222"/>
-      <c r="T4" s="222"/>
-      <c r="U4" s="222"/>
-      <c r="V4" s="222"/>
-      <c r="W4" s="222"/>
-      <c r="X4" s="222"/>
-      <c r="Y4" s="222"/>
-      <c r="Z4" s="222"/>
+      <c r="Q4" s="225"/>
+      <c r="R4" s="225"/>
+      <c r="S4" s="225"/>
+      <c r="T4" s="225"/>
+      <c r="U4" s="225"/>
+      <c r="V4" s="225"/>
+      <c r="W4" s="225"/>
+      <c r="X4" s="225"/>
+      <c r="Y4" s="225"/>
+      <c r="Z4" s="225"/>
       <c r="AB4" s="138" t="s">
         <v>202</v>
       </c>
@@ -29142,32 +29108,32 @@
       <c r="N8" s="91"/>
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="C9" s="219" t="s">
+      <c r="C9" s="222" t="s">
         <v>204</v>
       </c>
-      <c r="D9" s="219"/>
-      <c r="E9" s="219"/>
-      <c r="F9" s="219"/>
-      <c r="G9" s="219"/>
-      <c r="H9" s="219"/>
-      <c r="I9" s="219"/>
-      <c r="J9" s="219"/>
-      <c r="K9" s="219"/>
-      <c r="L9" s="219"/>
+      <c r="D9" s="222"/>
+      <c r="E9" s="222"/>
+      <c r="F9" s="222"/>
+      <c r="G9" s="222"/>
+      <c r="H9" s="222"/>
+      <c r="I9" s="222"/>
+      <c r="J9" s="222"/>
+      <c r="K9" s="222"/>
+      <c r="L9" s="222"/>
       <c r="N9" s="91"/>
-      <c r="P9" s="222" t="s">
+      <c r="P9" s="225" t="s">
         <v>209</v>
       </c>
-      <c r="Q9" s="222"/>
-      <c r="R9" s="222"/>
-      <c r="S9" s="222"/>
-      <c r="T9" s="222"/>
-      <c r="U9" s="222"/>
-      <c r="V9" s="222"/>
-      <c r="W9" s="222"/>
-      <c r="X9" s="222"/>
-      <c r="Y9" s="222"/>
-      <c r="Z9" s="222"/>
+      <c r="Q9" s="225"/>
+      <c r="R9" s="225"/>
+      <c r="S9" s="225"/>
+      <c r="T9" s="225"/>
+      <c r="U9" s="225"/>
+      <c r="V9" s="225"/>
+      <c r="W9" s="225"/>
+      <c r="X9" s="225"/>
+      <c r="Y9" s="225"/>
+      <c r="Z9" s="225"/>
       <c r="AB9" s="138" t="str">
         <f>AB4</f>
         <v>Q1-Q2-Q3</v>
@@ -29729,31 +29695,31 @@
       </c>
     </row>
     <row r="18" spans="2:26" x14ac:dyDescent="0.2">
-      <c r="C18" s="219" t="s">
+      <c r="C18" s="222" t="s">
         <v>207</v>
       </c>
-      <c r="D18" s="219"/>
-      <c r="E18" s="219"/>
-      <c r="F18" s="219"/>
-      <c r="G18" s="219"/>
-      <c r="H18" s="219"/>
-      <c r="I18" s="219"/>
-      <c r="J18" s="219"/>
-      <c r="K18" s="219"/>
-      <c r="L18" s="219"/>
-      <c r="P18" s="222" t="s">
+      <c r="D18" s="222"/>
+      <c r="E18" s="222"/>
+      <c r="F18" s="222"/>
+      <c r="G18" s="222"/>
+      <c r="H18" s="222"/>
+      <c r="I18" s="222"/>
+      <c r="J18" s="222"/>
+      <c r="K18" s="222"/>
+      <c r="L18" s="222"/>
+      <c r="P18" s="225" t="s">
         <v>207</v>
       </c>
-      <c r="Q18" s="222"/>
-      <c r="R18" s="222"/>
-      <c r="S18" s="222"/>
-      <c r="T18" s="222"/>
-      <c r="U18" s="222"/>
-      <c r="V18" s="222"/>
-      <c r="W18" s="222"/>
-      <c r="X18" s="222"/>
-      <c r="Y18" s="222"/>
-      <c r="Z18" s="222"/>
+      <c r="Q18" s="225"/>
+      <c r="R18" s="225"/>
+      <c r="S18" s="225"/>
+      <c r="T18" s="225"/>
+      <c r="U18" s="225"/>
+      <c r="V18" s="225"/>
+      <c r="W18" s="225"/>
+      <c r="X18" s="225"/>
+      <c r="Y18" s="225"/>
+      <c r="Z18" s="225"/>
     </row>
     <row r="19" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B19" s="7" t="s">
@@ -30238,20 +30204,20 @@
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A5" s="103"/>
-      <c r="C5" s="220" t="s">
+      <c r="C5" s="223" t="s">
         <v>168</v>
       </c>
-      <c r="D5" s="220"/>
-      <c r="E5" s="220"/>
-      <c r="F5" s="220"/>
-      <c r="G5" s="223"/>
-      <c r="H5" s="224" t="s">
+      <c r="D5" s="223"/>
+      <c r="E5" s="223"/>
+      <c r="F5" s="223"/>
+      <c r="G5" s="226"/>
+      <c r="H5" s="227" t="s">
         <v>169</v>
       </c>
-      <c r="I5" s="220"/>
-      <c r="J5" s="220"/>
-      <c r="K5" s="220"/>
-      <c r="L5" s="220"/>
+      <c r="I5" s="223"/>
+      <c r="J5" s="223"/>
+      <c r="K5" s="223"/>
+      <c r="L5" s="223"/>
       <c r="P5" s="228"/>
       <c r="Q5" s="228"/>
       <c r="R5" s="228"/>
@@ -30269,18 +30235,18 @@
     <row r="7" spans="1:28" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="108"/>
       <c r="B7" s="92"/>
-      <c r="C7" s="219" t="s">
+      <c r="C7" s="222" t="s">
         <v>178</v>
       </c>
-      <c r="D7" s="219"/>
-      <c r="E7" s="219"/>
-      <c r="F7" s="219"/>
-      <c r="G7" s="219"/>
-      <c r="H7" s="219"/>
-      <c r="I7" s="219"/>
-      <c r="J7" s="219"/>
-      <c r="K7" s="219"/>
-      <c r="L7" s="219"/>
+      <c r="D7" s="222"/>
+      <c r="E7" s="222"/>
+      <c r="F7" s="222"/>
+      <c r="G7" s="222"/>
+      <c r="H7" s="222"/>
+      <c r="I7" s="222"/>
+      <c r="J7" s="222"/>
+      <c r="K7" s="222"/>
+      <c r="L7" s="222"/>
       <c r="P7" s="228"/>
       <c r="Q7" s="228"/>
       <c r="R7" s="228"/>
@@ -30418,18 +30384,18 @@
       <c r="N11" s="91"/>
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="C12" s="219" t="s">
+      <c r="C12" s="222" t="s">
         <v>24</v>
       </c>
-      <c r="D12" s="219"/>
-      <c r="E12" s="219"/>
-      <c r="F12" s="219"/>
-      <c r="G12" s="219"/>
-      <c r="H12" s="219"/>
-      <c r="I12" s="219"/>
-      <c r="J12" s="219"/>
-      <c r="K12" s="219"/>
-      <c r="L12" s="219"/>
+      <c r="D12" s="222"/>
+      <c r="E12" s="222"/>
+      <c r="F12" s="222"/>
+      <c r="G12" s="222"/>
+      <c r="H12" s="222"/>
+      <c r="I12" s="222"/>
+      <c r="J12" s="222"/>
+      <c r="K12" s="222"/>
+      <c r="L12" s="222"/>
       <c r="N12" s="91"/>
       <c r="P12" s="228"/>
       <c r="Q12" s="228"/>
@@ -30743,18 +30709,18 @@
       <c r="D18" s="20"/>
     </row>
     <row r="20" spans="2:28" x14ac:dyDescent="0.2">
-      <c r="C20" s="219" t="s">
+      <c r="C20" s="222" t="s">
         <v>236</v>
       </c>
-      <c r="D20" s="219"/>
-      <c r="E20" s="219"/>
-      <c r="F20" s="219"/>
-      <c r="G20" s="219"/>
-      <c r="H20" s="219"/>
-      <c r="I20" s="219"/>
-      <c r="J20" s="219"/>
-      <c r="K20" s="219"/>
-      <c r="L20" s="219"/>
+      <c r="D20" s="222"/>
+      <c r="E20" s="222"/>
+      <c r="F20" s="222"/>
+      <c r="G20" s="222"/>
+      <c r="H20" s="222"/>
+      <c r="I20" s="222"/>
+      <c r="J20" s="222"/>
+      <c r="K20" s="222"/>
+      <c r="L20" s="222"/>
       <c r="P20" s="228"/>
       <c r="Q20" s="228"/>
       <c r="R20" s="228"/>
@@ -31020,18 +30986,18 @@
       </c>
     </row>
     <row r="30" spans="2:28" x14ac:dyDescent="0.2">
-      <c r="C30" s="219" t="s">
+      <c r="C30" s="222" t="s">
         <v>226</v>
       </c>
-      <c r="D30" s="219"/>
-      <c r="E30" s="219"/>
-      <c r="F30" s="219"/>
-      <c r="G30" s="219"/>
-      <c r="H30" s="219"/>
-      <c r="I30" s="219"/>
-      <c r="J30" s="219"/>
-      <c r="K30" s="219"/>
-      <c r="L30" s="219"/>
+      <c r="D30" s="222"/>
+      <c r="E30" s="222"/>
+      <c r="F30" s="222"/>
+      <c r="G30" s="222"/>
+      <c r="H30" s="222"/>
+      <c r="I30" s="222"/>
+      <c r="J30" s="222"/>
+      <c r="K30" s="222"/>
+      <c r="L30" s="222"/>
     </row>
     <row r="31" spans="2:28" x14ac:dyDescent="0.2">
       <c r="B31" s="7" t="s">
@@ -31259,10 +31225,10 @@
       </c>
     </row>
     <row r="37" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B37" s="220" t="s">
+      <c r="B37" s="223" t="s">
         <v>228</v>
       </c>
-      <c r="C37" s="220"/>
+      <c r="C37" s="223"/>
     </row>
     <row r="38" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B38" s="1" t="s">
@@ -31282,13 +31248,13 @@
     </row>
     <row r="42" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B42" s="7"/>
-      <c r="C42" s="220" t="s">
+      <c r="C42" s="223" t="s">
         <v>227</v>
       </c>
-      <c r="D42" s="220"/>
-      <c r="E42" s="220"/>
-      <c r="F42" s="220"/>
-      <c r="G42" s="220"/>
+      <c r="D42" s="223"/>
+      <c r="E42" s="223"/>
+      <c r="F42" s="223"/>
+      <c r="G42" s="223"/>
     </row>
     <row r="43" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B43" s="7" t="s">
@@ -31418,10 +31384,10 @@
       </c>
     </row>
     <row r="50" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B50" s="220" t="s">
+      <c r="B50" s="223" t="s">
         <v>232</v>
       </c>
-      <c r="C50" s="220"/>
+      <c r="C50" s="223"/>
     </row>
     <row r="51" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B51" s="1" t="s">

</xml_diff>